<commit_message>
Load real 2026-2027 Shala schedule into calendar (from base Excel sheet)
</commit_message>
<xml_diff>
--- a/data/shala-calendar.xlsx
+++ b/data/shala-calendar.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shala Calendar" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,6 +40,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0056127D"/>
+        <bgColor rgb="0056127D"/>
       </patternFill>
     </fill>
   </fills>
@@ -423,16 +424,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,11 +483,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -494,14 +495,10 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Level 1-3 batches, virtual</t>
+          <t>Online · Week 1</t>
         </is>
       </c>
     </row>
@@ -511,15 +508,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -527,12 +524,12 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Online · Week 2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -540,15 +537,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -556,12 +553,12 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Online · Week 3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -569,15 +566,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -585,12 +582,12 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Online · Week 4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -598,26 +595,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No Class - Labor Day Weekend</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Holiday</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Enjoy the long weekend!</t>
+          <t>Online · Week 5</t>
         </is>
       </c>
     </row>
@@ -627,15 +624,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Shala Reopens - First Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -643,14 +640,10 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>New academic year begins</t>
+          <t>Online · Week 6</t>
         </is>
       </c>
     </row>
@@ -660,15 +653,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -676,12 +669,12 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Online · Week 7</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -689,15 +682,15 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -705,12 +698,12 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Online · Week 8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -718,27 +711,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Dasara</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -751,11 +740,11 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Marathi Shala Class</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -763,12 +752,12 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Online · Week 9</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -776,26 +765,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bhondla &amp; Kanya Pujan (in-person)</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Event</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Combined with Mandal event - attendance counts toward grading</t>
+          <t>Online · Week 10</t>
         </is>
       </c>
     </row>
@@ -805,24 +794,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>No Class - Diwali Break</t>
+          <t>Diwali</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Holiday</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -834,22 +827,1633 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mid-Term Exam Window Opens</t>
+          <t>Marathi Shala</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Exam</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Speak with your class teacher to schedule</t>
+          <t>Online · Week 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Online · Week 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>23</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Online · Week 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>27</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Online · Week 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>7</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Online · Week 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>13</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>14</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Online · Week 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>19</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>20</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>21</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Online · Week 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>24</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>25</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>26</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>27</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>28</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>29</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>30</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>31</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Christmas &amp; New Year Break</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Online · Week 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>11</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Online · Week 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>18</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>MLK Day</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>19</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Online · Week 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>25</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Online · Week 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Online · Week 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Online · Week 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>15</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Winter Break</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>16</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Winter Break</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>17</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Winter Break</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>18</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Winter Break</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>19</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Winter Break</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>22</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Online · Week 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Online · Week 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>8</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Online · Week 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>15</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Online · Week 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>22</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Online · Week 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>26</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Good Friday</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>29</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Online · Week 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>5</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Online · Week 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>10</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Gudhi Padwa</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>12</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Online · Week 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>19</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Spring Break</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>20</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Spring Break</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>21</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Spring Break</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>22</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Spring Break</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>23</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Spring Break</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>26</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Online · Week 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>3</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Online · Week 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>10</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Marathi Shala</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Online · Week 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>15</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>16</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>22</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>23</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>6</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Picnic</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>13</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Picnic (rain date)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>In-person</t>
         </is>
       </c>
     </row>

</xml_diff>